<commit_message>
Add test cases and automate create user api
</commit_message>
<xml_diff>
--- a/manual/API Test Cases.xlsx
+++ b/manual/API Test Cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zia kayani\Documents\automationexercise\manual\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B806A33F-7443-4388-AC35-FAA3731C1BA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC44F6DF-CE33-4E87-B74D-B27E56BC480B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{F8B6A9C3-3DD6-41E1-BE41-0189C9C242F4}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="102">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -125,9 +125,6 @@
     <t>TC014</t>
   </si>
   <si>
-    <t>TC015</t>
-  </si>
-  <si>
     <t>TC016</t>
   </si>
   <si>
@@ -138,9 +135,6 @@
   </si>
   <si>
     <t>TC019</t>
-  </si>
-  <si>
-    <t>TC020</t>
   </si>
   <si>
     <r>
@@ -219,6 +213,195 @@
   </si>
   <si>
     <t>API</t>
+  </si>
+  <si>
+    <t>Products API</t>
+  </si>
+  <si>
+    <t>Get all products list</t>
+  </si>
+  <si>
+    <t>API is up</t>
+  </si>
+  <si>
+    <t>Send GET request to /api/productsList</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>Status 200 and products list returned</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Major</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>POST not allowed on products list</t>
+  </si>
+  <si>
+    <t>Negative API</t>
+  </si>
+  <si>
+    <t>Send POST request to /api/productsList</t>
+  </si>
+  <si>
+    <t>Status 405 with error message</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>Minor</t>
+  </si>
+  <si>
+    <t>Brands API</t>
+  </si>
+  <si>
+    <t>Get all brands list</t>
+  </si>
+  <si>
+    <t>Send GET request to /api/brandsList</t>
+  </si>
+  <si>
+    <t>Status 200 and brands list returned</t>
+  </si>
+  <si>
+    <t>PUT not allowed on brands list</t>
+  </si>
+  <si>
+    <t>Send PUT request to /api/brandsList</t>
+  </si>
+  <si>
+    <t>Status 405 error</t>
+  </si>
+  <si>
+    <t>Search API</t>
+  </si>
+  <si>
+    <t>Search product with valid input</t>
+  </si>
+  <si>
+    <t>Send POST request to /api/searchProduct</t>
+  </si>
+  <si>
+    <t>search_product=tshirt</t>
+  </si>
+  <si>
+    <t>Status 200 and matching products returned</t>
+  </si>
+  <si>
+    <t>Search product without parameter</t>
+  </si>
+  <si>
+    <t>Send POST without search_product</t>
+  </si>
+  <si>
+    <t>Status 400 bad request</t>
+  </si>
+  <si>
+    <t>Auth API</t>
+  </si>
+  <si>
+    <t>Login with valid credentials</t>
+  </si>
+  <si>
+    <t>User exists</t>
+  </si>
+  <si>
+    <t>Send POST to /api/verifyLogin</t>
+  </si>
+  <si>
+    <t>email, password valid</t>
+  </si>
+  <si>
+    <t>Status 200 User exists</t>
+  </si>
+  <si>
+    <t>Critical</t>
+  </si>
+  <si>
+    <t>Login without email</t>
+  </si>
+  <si>
+    <t>Send POST with only password</t>
+  </si>
+  <si>
+    <t>password only</t>
+  </si>
+  <si>
+    <t>DELETE method not allowed on login</t>
+  </si>
+  <si>
+    <t>Send DELETE request to /api/verifyLogin</t>
+  </si>
+  <si>
+    <t>Login with invalid credentials</t>
+  </si>
+  <si>
+    <t>Send POST with invalid email/password</t>
+  </si>
+  <si>
+    <t>invalid credentials</t>
+  </si>
+  <si>
+    <t>Status 404 user not found</t>
+  </si>
+  <si>
+    <t>User API</t>
+  </si>
+  <si>
+    <t>Create new user account</t>
+  </si>
+  <si>
+    <t>Send POST to /api/createAccount</t>
+  </si>
+  <si>
+    <t>Full valid user data</t>
+  </si>
+  <si>
+    <t>Status 201 user created</t>
+  </si>
+  <si>
+    <t>Delete user account</t>
+  </si>
+  <si>
+    <t>Send DELETE to /api/deleteAccount</t>
+  </si>
+  <si>
+    <t>email, password</t>
+  </si>
+  <si>
+    <t>Status 200 account deleted</t>
+  </si>
+  <si>
+    <t>Update user account</t>
+  </si>
+  <si>
+    <t>Send PUT to /api/updateAccount</t>
+  </si>
+  <si>
+    <t>Updated user data</t>
+  </si>
+  <si>
+    <t>Status 200 user updated</t>
+  </si>
+  <si>
+    <t>Get user detail by email</t>
+  </si>
+  <si>
+    <t>Send GET to /api/getUserDetailByEmail</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>Status 200 with user details</t>
   </si>
 </sst>
 </file>
@@ -283,7 +466,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -300,6 +483,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -309,7 +507,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -652,22 +850,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE27A1CA-9D95-4D98-A36F-CCCABFF34EA0}">
-  <dimension ref="A1:O27"/>
+  <dimension ref="A1:O25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.21875" customWidth="1"/>
-    <col min="3" max="3" width="17.21875" customWidth="1"/>
+    <col min="2" max="2" width="13.33203125" customWidth="1"/>
+    <col min="3" max="3" width="32.6640625" customWidth="1"/>
     <col min="4" max="4" width="18.77734375" customWidth="1"/>
-    <col min="8" max="8" width="12.21875" customWidth="1"/>
+    <col min="5" max="5" width="23.44140625" customWidth="1"/>
+    <col min="6" max="6" width="37.33203125" customWidth="1"/>
+    <col min="7" max="7" width="21" customWidth="1"/>
+    <col min="8" max="8" width="38.6640625" customWidth="1"/>
+    <col min="9" max="9" width="14.33203125" customWidth="1"/>
     <col min="10" max="10" width="22" customWidth="1"/>
     <col min="11" max="11" width="17.109375" customWidth="1"/>
     <col min="13" max="13" width="16.6640625" customWidth="1"/>
-    <col min="14" max="14" width="11" customWidth="1"/>
+    <col min="14" max="14" width="27.33203125" customWidth="1"/>
+    <col min="15" max="15" width="25.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -678,7 +882,7 @@
     </row>
     <row r="2" spans="1:15" ht="18" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -689,7 +893,7 @@
     </row>
     <row r="3" spans="1:15" ht="18" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -700,7 +904,7 @@
     </row>
     <row r="4" spans="1:15" ht="18" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -711,7 +915,7 @@
     </row>
     <row r="5" spans="1:15" ht="18" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -720,7 +924,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="7" spans="1:15" s="3" customFormat="1" ht="52.8" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:15" s="3" customFormat="1" ht="52.2" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>0</v>
       </c>
@@ -767,125 +971,518 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:15" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>15</v>
       </c>
+      <c r="B8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C8" t="s">
+        <v>40</v>
+      </c>
       <c r="D8" t="s">
-        <v>40</v>
+        <v>38</v>
+      </c>
+      <c r="E8" t="s">
+        <v>41</v>
+      </c>
+      <c r="F8" t="s">
+        <v>42</v>
+      </c>
+      <c r="G8" t="s">
+        <v>43</v>
+      </c>
+      <c r="H8" t="s">
+        <v>44</v>
+      </c>
+      <c r="J8" t="s">
+        <v>45</v>
+      </c>
+      <c r="K8" t="s">
+        <v>46</v>
+      </c>
+      <c r="M8" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>16</v>
       </c>
+      <c r="B9" t="s">
+        <v>39</v>
+      </c>
+      <c r="C9" t="s">
+        <v>48</v>
+      </c>
+      <c r="D9" t="s">
+        <v>49</v>
+      </c>
+      <c r="E9" t="s">
+        <v>41</v>
+      </c>
+      <c r="F9" t="s">
+        <v>50</v>
+      </c>
+      <c r="G9" t="s">
+        <v>43</v>
+      </c>
+      <c r="H9" t="s">
+        <v>51</v>
+      </c>
+      <c r="J9" t="s">
+        <v>52</v>
+      </c>
+      <c r="K9" t="s">
+        <v>53</v>
+      </c>
+      <c r="M9" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>17</v>
       </c>
+      <c r="B10" t="s">
+        <v>54</v>
+      </c>
+      <c r="C10" t="s">
+        <v>55</v>
+      </c>
+      <c r="D10" t="s">
+        <v>38</v>
+      </c>
+      <c r="E10" t="s">
+        <v>41</v>
+      </c>
+      <c r="F10" t="s">
+        <v>56</v>
+      </c>
+      <c r="G10" t="s">
+        <v>43</v>
+      </c>
+      <c r="H10" t="s">
+        <v>57</v>
+      </c>
+      <c r="J10" t="s">
+        <v>45</v>
+      </c>
+      <c r="K10" t="s">
+        <v>46</v>
+      </c>
+      <c r="M10" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>18</v>
       </c>
+      <c r="B11" t="s">
+        <v>54</v>
+      </c>
+      <c r="C11" t="s">
+        <v>58</v>
+      </c>
+      <c r="D11" t="s">
+        <v>49</v>
+      </c>
+      <c r="E11" t="s">
+        <v>41</v>
+      </c>
+      <c r="F11" t="s">
+        <v>59</v>
+      </c>
+      <c r="G11" t="s">
+        <v>43</v>
+      </c>
+      <c r="H11" t="s">
+        <v>60</v>
+      </c>
+      <c r="J11" t="s">
+        <v>52</v>
+      </c>
+      <c r="K11" t="s">
+        <v>53</v>
+      </c>
+      <c r="M11" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>19</v>
       </c>
+      <c r="B12" t="s">
+        <v>61</v>
+      </c>
+      <c r="C12" t="s">
+        <v>62</v>
+      </c>
+      <c r="D12" t="s">
+        <v>38</v>
+      </c>
+      <c r="E12" t="s">
+        <v>41</v>
+      </c>
+      <c r="F12" t="s">
+        <v>63</v>
+      </c>
+      <c r="G12" t="s">
+        <v>64</v>
+      </c>
+      <c r="H12" t="s">
+        <v>65</v>
+      </c>
+      <c r="J12" t="s">
+        <v>45</v>
+      </c>
+      <c r="K12" t="s">
+        <v>46</v>
+      </c>
+      <c r="M12" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>20</v>
       </c>
+      <c r="B13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C13" t="s">
+        <v>66</v>
+      </c>
+      <c r="D13" t="s">
+        <v>49</v>
+      </c>
+      <c r="E13" t="s">
+        <v>41</v>
+      </c>
+      <c r="F13" t="s">
+        <v>67</v>
+      </c>
+      <c r="G13" t="s">
+        <v>43</v>
+      </c>
+      <c r="H13" t="s">
+        <v>68</v>
+      </c>
+      <c r="J13" t="s">
+        <v>45</v>
+      </c>
+      <c r="K13" t="s">
+        <v>46</v>
+      </c>
+      <c r="M13" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>21</v>
       </c>
+      <c r="B14" t="s">
+        <v>69</v>
+      </c>
+      <c r="C14" t="s">
+        <v>70</v>
+      </c>
+      <c r="D14" t="s">
+        <v>38</v>
+      </c>
+      <c r="E14" t="s">
+        <v>71</v>
+      </c>
+      <c r="F14" t="s">
+        <v>72</v>
+      </c>
+      <c r="G14" t="s">
+        <v>73</v>
+      </c>
+      <c r="H14" t="s">
+        <v>74</v>
+      </c>
+      <c r="J14" t="s">
+        <v>45</v>
+      </c>
+      <c r="K14" t="s">
+        <v>75</v>
+      </c>
+      <c r="M14" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>22</v>
       </c>
+      <c r="B15" t="s">
+        <v>69</v>
+      </c>
+      <c r="C15" t="s">
+        <v>76</v>
+      </c>
+      <c r="D15" t="s">
+        <v>49</v>
+      </c>
+      <c r="E15" t="s">
+        <v>41</v>
+      </c>
+      <c r="F15" t="s">
+        <v>77</v>
+      </c>
+      <c r="G15" t="s">
+        <v>78</v>
+      </c>
+      <c r="H15" t="s">
+        <v>68</v>
+      </c>
+      <c r="J15" t="s">
+        <v>45</v>
+      </c>
+      <c r="K15" t="s">
+        <v>46</v>
+      </c>
+      <c r="M15" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B16" t="s">
+        <v>69</v>
+      </c>
+      <c r="C16" t="s">
+        <v>79</v>
+      </c>
+      <c r="D16" t="s">
+        <v>49</v>
+      </c>
+      <c r="E16" t="s">
+        <v>41</v>
+      </c>
+      <c r="F16" t="s">
+        <v>80</v>
+      </c>
+      <c r="G16" t="s">
+        <v>43</v>
+      </c>
+      <c r="H16" t="s">
+        <v>60</v>
+      </c>
+      <c r="J16" t="s">
+        <v>52</v>
+      </c>
+      <c r="K16" t="s">
+        <v>53</v>
+      </c>
+      <c r="M16" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B17" t="s">
+        <v>69</v>
+      </c>
+      <c r="C17" t="s">
+        <v>81</v>
+      </c>
+      <c r="D17" t="s">
+        <v>49</v>
+      </c>
+      <c r="E17" t="s">
+        <v>41</v>
+      </c>
+      <c r="F17" t="s">
+        <v>82</v>
+      </c>
+      <c r="G17" t="s">
+        <v>83</v>
+      </c>
+      <c r="H17" t="s">
+        <v>84</v>
+      </c>
+      <c r="J17" t="s">
+        <v>45</v>
+      </c>
+      <c r="K17" t="s">
+        <v>46</v>
+      </c>
+      <c r="M17" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B18" t="s">
+        <v>85</v>
+      </c>
+      <c r="C18" t="s">
+        <v>86</v>
+      </c>
+      <c r="D18" t="s">
+        <v>38</v>
+      </c>
+      <c r="E18" t="s">
+        <v>41</v>
+      </c>
+      <c r="F18" t="s">
+        <v>87</v>
+      </c>
+      <c r="G18" t="s">
+        <v>88</v>
+      </c>
+      <c r="H18" t="s">
+        <v>89</v>
+      </c>
+      <c r="J18" t="s">
+        <v>45</v>
+      </c>
+      <c r="K18" t="s">
+        <v>75</v>
+      </c>
+      <c r="M18" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B19" t="s">
+        <v>85</v>
+      </c>
+      <c r="C19" t="s">
+        <v>90</v>
+      </c>
+      <c r="D19" t="s">
+        <v>38</v>
+      </c>
+      <c r="E19" t="s">
+        <v>71</v>
+      </c>
+      <c r="F19" t="s">
+        <v>91</v>
+      </c>
+      <c r="G19" t="s">
+        <v>92</v>
+      </c>
+      <c r="H19" t="s">
+        <v>93</v>
+      </c>
+      <c r="J19" t="s">
+        <v>45</v>
+      </c>
+      <c r="K19" t="s">
+        <v>75</v>
+      </c>
+      <c r="M19" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B20" t="s">
+        <v>85</v>
+      </c>
+      <c r="C20" t="s">
+        <v>94</v>
+      </c>
+      <c r="D20" t="s">
+        <v>38</v>
+      </c>
+      <c r="E20" t="s">
+        <v>71</v>
+      </c>
+      <c r="F20" t="s">
+        <v>95</v>
+      </c>
+      <c r="G20" t="s">
+        <v>96</v>
+      </c>
+      <c r="H20" t="s">
+        <v>97</v>
+      </c>
+      <c r="J20" t="s">
+        <v>45</v>
+      </c>
+      <c r="K20" t="s">
+        <v>46</v>
+      </c>
+      <c r="M20" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B21" t="s">
+        <v>85</v>
+      </c>
+      <c r="C21" t="s">
+        <v>98</v>
+      </c>
+      <c r="D21" t="s">
+        <v>38</v>
+      </c>
+      <c r="E21" t="s">
+        <v>71</v>
+      </c>
+      <c r="F21" t="s">
+        <v>99</v>
+      </c>
+      <c r="G21" t="s">
+        <v>100</v>
+      </c>
+      <c r="H21" t="s">
+        <v>101</v>
+      </c>
+      <c r="J21" t="s">
+        <v>45</v>
+      </c>
+      <c r="K21" t="s">
+        <v>46</v>
+      </c>
+      <c r="M21" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>34</v>
-      </c>
-    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
-  <dataValidations count="4">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D8" xr:uid="{19FD72A4-C721-4F10-B04E-1A777D0A4528}">
-      <formula1>"UI,Functional,API,"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J8" xr:uid="{FFB2E585-237F-4F82-8E4D-B4703CA95639}">
-      <formula1>"high,medium,low"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K8" xr:uid="{F9B926B2-83B6-4A83-BAA5-BF781BDAE6D4}">
-      <formula1>"critical,major,minor"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L8" xr:uid="{185A1577-949E-48AF-BF2B-284486DC38DC}">
-      <formula1>"pass,fail"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updated test cases sheet
</commit_message>
<xml_diff>
--- a/manual/API Test Cases.xlsx
+++ b/manual/API Test Cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zia kayani\Documents\automationexercise\manual\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC44F6DF-CE33-4E87-B74D-B27E56BC480B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F560D4C-1E8C-4E61-BD92-AEE6A0E3F932}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{F8B6A9C3-3DD6-41E1-BE41-0189C9C242F4}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="113">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -402,6 +402,39 @@
   </si>
   <si>
     <t>Status 200 with user details</t>
+  </si>
+  <si>
+    <t>Status 200 user updated`</t>
+  </si>
+  <si>
+    <t>pass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test script passed and api works in postman </t>
+  </si>
+  <si>
+    <t>tests/test_user.py//test_login_user_with_valid_data</t>
+  </si>
+  <si>
+    <t>tests/test_user.py//test_login_user_without_email</t>
+  </si>
+  <si>
+    <t>tests/test_user.py// test_login_user_with_delete_method</t>
+  </si>
+  <si>
+    <t>tests/test_user.py//test_login_user_with_invalid_data</t>
+  </si>
+  <si>
+    <t>tests/test_user.py//test_create_new_user</t>
+  </si>
+  <si>
+    <t>tests/test_user.py//test_delete_user</t>
+  </si>
+  <si>
+    <t>tests/test_user.py//test_update_user_details</t>
+  </si>
+  <si>
+    <t>tests/test_user.py//test_get_user_details</t>
   </si>
 </sst>
 </file>
@@ -861,12 +894,12 @@
     <col min="6" max="6" width="37.33203125" customWidth="1"/>
     <col min="7" max="7" width="21" customWidth="1"/>
     <col min="8" max="8" width="38.6640625" customWidth="1"/>
-    <col min="9" max="9" width="14.33203125" customWidth="1"/>
+    <col min="9" max="9" width="35.77734375" customWidth="1"/>
     <col min="10" max="10" width="22" customWidth="1"/>
     <col min="11" max="11" width="17.109375" customWidth="1"/>
     <col min="13" max="13" width="16.6640625" customWidth="1"/>
-    <col min="14" max="14" width="27.33203125" customWidth="1"/>
-    <col min="15" max="15" width="25.6640625" customWidth="1"/>
+    <col min="14" max="14" width="41.109375" customWidth="1"/>
+    <col min="15" max="15" width="36.88671875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="18" x14ac:dyDescent="0.35">
@@ -1206,14 +1239,26 @@
       <c r="H14" t="s">
         <v>74</v>
       </c>
+      <c r="I14" t="s">
+        <v>74</v>
+      </c>
       <c r="J14" t="s">
         <v>45</v>
       </c>
       <c r="K14" t="s">
         <v>75</v>
       </c>
+      <c r="L14" t="s">
+        <v>103</v>
+      </c>
       <c r="M14" t="s">
         <v>47</v>
+      </c>
+      <c r="N14" t="s">
+        <v>105</v>
+      </c>
+      <c r="O14" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
@@ -1241,14 +1286,26 @@
       <c r="H15" t="s">
         <v>68</v>
       </c>
+      <c r="I15" t="s">
+        <v>68</v>
+      </c>
       <c r="J15" t="s">
         <v>45</v>
       </c>
       <c r="K15" t="s">
         <v>46</v>
       </c>
+      <c r="L15" t="s">
+        <v>103</v>
+      </c>
       <c r="M15" t="s">
         <v>47</v>
+      </c>
+      <c r="N15" t="s">
+        <v>106</v>
+      </c>
+      <c r="O15" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
@@ -1276,17 +1333,29 @@
       <c r="H16" t="s">
         <v>60</v>
       </c>
+      <c r="I16" t="s">
+        <v>60</v>
+      </c>
       <c r="J16" t="s">
         <v>52</v>
       </c>
       <c r="K16" t="s">
         <v>53</v>
       </c>
+      <c r="L16" t="s">
+        <v>103</v>
+      </c>
       <c r="M16" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="N16" t="s">
+        <v>107</v>
+      </c>
+      <c r="O16" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>24</v>
       </c>
@@ -1311,17 +1380,29 @@
       <c r="H17" t="s">
         <v>84</v>
       </c>
+      <c r="I17" t="s">
+        <v>84</v>
+      </c>
       <c r="J17" t="s">
         <v>45</v>
       </c>
       <c r="K17" t="s">
         <v>46</v>
       </c>
+      <c r="L17" t="s">
+        <v>103</v>
+      </c>
       <c r="M17" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="N17" t="s">
+        <v>108</v>
+      </c>
+      <c r="O17" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>25</v>
       </c>
@@ -1346,17 +1427,29 @@
       <c r="H18" t="s">
         <v>89</v>
       </c>
+      <c r="I18" t="s">
+        <v>89</v>
+      </c>
       <c r="J18" t="s">
         <v>45</v>
       </c>
       <c r="K18" t="s">
         <v>75</v>
       </c>
+      <c r="L18" t="s">
+        <v>103</v>
+      </c>
       <c r="M18" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="N18" t="s">
+        <v>109</v>
+      </c>
+      <c r="O18" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>26</v>
       </c>
@@ -1381,17 +1474,29 @@
       <c r="H19" t="s">
         <v>93</v>
       </c>
+      <c r="I19" t="s">
+        <v>93</v>
+      </c>
       <c r="J19" t="s">
         <v>45</v>
       </c>
       <c r="K19" t="s">
         <v>75</v>
       </c>
+      <c r="L19" t="s">
+        <v>103</v>
+      </c>
       <c r="M19" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="N19" t="s">
+        <v>110</v>
+      </c>
+      <c r="O19" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>27</v>
       </c>
@@ -1414,6 +1519,9 @@
         <v>96</v>
       </c>
       <c r="H20" t="s">
+        <v>102</v>
+      </c>
+      <c r="I20" t="s">
         <v>97</v>
       </c>
       <c r="J20" t="s">
@@ -1422,11 +1530,20 @@
       <c r="K20" t="s">
         <v>46</v>
       </c>
+      <c r="L20" t="s">
+        <v>103</v>
+      </c>
       <c r="M20" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="N20" t="s">
+        <v>111</v>
+      </c>
+      <c r="O20" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>28</v>
       </c>
@@ -1451,32 +1568,44 @@
       <c r="H21" t="s">
         <v>101</v>
       </c>
+      <c r="I21" t="s">
+        <v>101</v>
+      </c>
       <c r="J21" t="s">
         <v>45</v>
       </c>
       <c r="K21" t="s">
         <v>46</v>
       </c>
+      <c r="L21" t="s">
+        <v>103</v>
+      </c>
       <c r="M21" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="N21" t="s">
+        <v>112</v>
+      </c>
+      <c r="O21" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>32</v>
       </c>

</xml_diff>

<commit_message>
update test cases document
</commit_message>
<xml_diff>
--- a/manual/API Test Cases.xlsx
+++ b/manual/API Test Cases.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zia kayani\Documents\automationexercise\manual\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F560D4C-1E8C-4E61-BD92-AEE6A0E3F932}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4490F32D-48CB-4D8A-9E01-AD7B8FB2F10C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{F8B6A9C3-3DD6-41E1-BE41-0189C9C242F4}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="119">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -435,6 +435,24 @@
   </si>
   <si>
     <t>tests/test_user.py//test_get_user_details</t>
+  </si>
+  <si>
+    <t>tests/test_product.py/ test_get_all_products_list</t>
+  </si>
+  <si>
+    <t>tests/test_product.py/test_post_to_all_product_list</t>
+  </si>
+  <si>
+    <t>tests/test_product.py/test_get_all_brands</t>
+  </si>
+  <si>
+    <t>tests/test_product.py/test_put_to_all_brands</t>
+  </si>
+  <si>
+    <t>tests/test_product.py/test_search_a_product</t>
+  </si>
+  <si>
+    <t>tests/test_product.py/test_search_a_product_without_payload</t>
   </si>
 </sst>
 </file>
@@ -898,7 +916,7 @@
     <col min="10" max="10" width="22" customWidth="1"/>
     <col min="11" max="11" width="17.109375" customWidth="1"/>
     <col min="13" max="13" width="16.6640625" customWidth="1"/>
-    <col min="14" max="14" width="41.109375" customWidth="1"/>
+    <col min="14" max="14" width="52.44140625" customWidth="1"/>
     <col min="15" max="15" width="36.88671875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1029,14 +1047,26 @@
       <c r="H8" t="s">
         <v>44</v>
       </c>
+      <c r="I8" t="s">
+        <v>44</v>
+      </c>
       <c r="J8" t="s">
         <v>45</v>
       </c>
       <c r="K8" t="s">
         <v>46</v>
       </c>
+      <c r="L8" t="s">
+        <v>103</v>
+      </c>
       <c r="M8" t="s">
         <v>47</v>
+      </c>
+      <c r="N8" t="s">
+        <v>113</v>
+      </c>
+      <c r="O8" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
@@ -1064,14 +1094,26 @@
       <c r="H9" t="s">
         <v>51</v>
       </c>
+      <c r="I9" t="s">
+        <v>51</v>
+      </c>
       <c r="J9" t="s">
         <v>52</v>
       </c>
       <c r="K9" t="s">
         <v>53</v>
       </c>
+      <c r="L9" t="s">
+        <v>103</v>
+      </c>
       <c r="M9" t="s">
         <v>47</v>
+      </c>
+      <c r="N9" t="s">
+        <v>114</v>
+      </c>
+      <c r="O9" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
@@ -1099,14 +1141,26 @@
       <c r="H10" t="s">
         <v>57</v>
       </c>
+      <c r="I10" t="s">
+        <v>57</v>
+      </c>
       <c r="J10" t="s">
         <v>45</v>
       </c>
       <c r="K10" t="s">
         <v>46</v>
       </c>
+      <c r="L10" t="s">
+        <v>103</v>
+      </c>
       <c r="M10" t="s">
         <v>47</v>
+      </c>
+      <c r="N10" t="s">
+        <v>115</v>
+      </c>
+      <c r="O10" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
@@ -1134,14 +1188,26 @@
       <c r="H11" t="s">
         <v>60</v>
       </c>
+      <c r="I11" t="s">
+        <v>60</v>
+      </c>
       <c r="J11" t="s">
         <v>52</v>
       </c>
       <c r="K11" t="s">
         <v>53</v>
       </c>
+      <c r="L11" t="s">
+        <v>103</v>
+      </c>
       <c r="M11" t="s">
         <v>47</v>
+      </c>
+      <c r="N11" t="s">
+        <v>116</v>
+      </c>
+      <c r="O11" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
@@ -1169,14 +1235,26 @@
       <c r="H12" t="s">
         <v>65</v>
       </c>
+      <c r="I12" t="s">
+        <v>65</v>
+      </c>
       <c r="J12" t="s">
         <v>45</v>
       </c>
       <c r="K12" t="s">
         <v>46</v>
       </c>
+      <c r="L12" t="s">
+        <v>103</v>
+      </c>
       <c r="M12" t="s">
         <v>47</v>
+      </c>
+      <c r="N12" t="s">
+        <v>117</v>
+      </c>
+      <c r="O12" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
@@ -1204,14 +1282,26 @@
       <c r="H13" t="s">
         <v>68</v>
       </c>
+      <c r="I13" t="s">
+        <v>68</v>
+      </c>
       <c r="J13" t="s">
         <v>45</v>
       </c>
       <c r="K13" t="s">
         <v>46</v>
       </c>
+      <c r="L13" t="s">
+        <v>103</v>
+      </c>
       <c r="M13" t="s">
         <v>47</v>
+      </c>
+      <c r="N13" t="s">
+        <v>118</v>
+      </c>
+      <c r="O13" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">

</xml_diff>